<commit_message>
docs(nghien-cuu): 03 Excel mau thuan san xuat gom theo cau hoi that — 16 cau, y kien ai noi gi, AI de nghi, o tra loi
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/erp/nghien-cuu/03-mau-thuan-san-xuat.xlsx
+++ b/doc/erp/nghien-cuu/03-mau-thuan-san-xuat.xlsx
@@ -7,11 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mâu thuẫn" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Câu hỏi cần chốt" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Mâu thuẫn'!$A$1:$F$26</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -451,14 +449,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
     <col width="40" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -475,65 +473,64 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Số câu trả lời mâu thuẫn</t>
+          <t>Số ý kiến khác nhau</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Các câu trả lời mâu thuẫn</t>
+          <t>Các ý kiến (ai nói gì)</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>AI hỗ trợ ra quyết định</t>
+          <t>AI đề nghị</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Trả lời của Sản xuất</t>
+          <t>Sản xuất trả lời (chọn ý kiến số mấy, hoặc ghi cách khác)</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>M01</t>
-        </is>
+      <c r="A2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng?</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>- [Suy diễn (AI) · Chuyên viên Điều phối vật tư bao bì · V4 · C1] Trưởng phòng sản xuất (khi các phương án kiểm tra tồn kho luân chuyển nội bộ, thương lượng Kinh doanh dời ngày và trao đổi Thu mua mua hàng không giải quyết được)
-- [Trưởng nhóm Quản lý dữ liệu · V6 · C1] Phòng Kinh doanh là đơn vị xem xét và quyết định việc tiếp tục triển khai hoặc tạm dừng đơn hàng khi kiểm tra điều kiện có vướng mắc; Điều phối thành phẩm phối hợp kiểm tra và thông báo</t>
+          <t>1. Trưởng phòng sản xuất (khi các phương án kiểm tra tồn kho luân chuyển nội bộ, thương lượng Kinh doanh dời ngày và trao đổi Thu mua mua hàng không giải quyết được)  (AI suy ra từ Chuyên viên Điều phối vật tư bao bì)
+2. Phòng Kinh doanh là đơn vị xem xét và quyết định việc tiếp tục triển khai hoặc tạm dừng đơn hàng khi kiểm tra điều kiện có vướng mắc; Điều phối thành phẩm phối hợp kiểm tra và thông báo  (Trưởng nhóm Quản lý dữ liệu)
+3. Trưởng phòng (Quản lý sản xuất) chịu trách nhiệm cuối quyết định duyệt cho đơn hàng triển khai (kể cả trường hợp duyệt trước bổ sung sau)  (Chị Ngân)
+4. Quản lý sản xuất là người quyết định cuối cùng (cho duyệt trước bổ sung sau hoặc tạm ngưng đơn) dựa trên dữ liệu kiểm tra từ các nhóm nội bộ; Trưởng nhóm Điều phối cập nhật tiến độ lại cho Kinh doanh  (Trưởng nhóm Điều phối)
+5. Trưởng phòng sản xuất hoặc Phòng Kinh doanh quyết định cuối cùng về việc duyệt tiếp hay dừng đơn khi tồn kho VTBB không đủ hoặc không kịp tiến độ đơn hàng  (Chuyên viên Điều phối vật tư bao bì)
+6. Phòng Kinh doanh xem xét và quyết định phương án duyệt hoặc hoãn đơn hàng khi NL/BTP không đủ hoặc không kịp tiến độ  (Chuyên viên Điều phối nguyên liệu/bán thành phẩm)
+7. Nhân sự phụ trách thông báo trực tiếp cho Phòng Kinh doanh và Quản lý để xem xét, quyết định tiếp tục triển khai hoặc tạm dừng đơn hàng khi điều kiện triển khai chưa đáp ứng  (Trưởng nhóm Quản lý dữ liệu)
+8. Quản lý sản xuất là người quyết định cuối cùng việc duyệt cho đơn hàng triển khai hay không khi hồ sơ pháp lý chưa đạt hoặc chưa đủ  (Chuyên viên Pháp lý - Xử lý sự cố)</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Nguồn A là giả thuyết MIC suy ra từ câu trả lời, chưa được người trả lời xác nhận (độ tin thấp). Nguồn B là as-is, độ tin cao. Nhận định MIC: thiếu VTBB thì lần lượt luân chuyển nội bộ, xin KD dời ngày, nhờ Thu mua mua thêm; không xong mới trình Trưởng phòng. Nguồn B nói KD quyết.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
+Người nên chốt: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
         </is>
       </c>
       <c r="F2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>M02</t>
-        </is>
+      <c r="A3" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Phiếu yêu cầu điều chuyển nguyên liệu gửi cho ai, và ai là đầu mối làm việc với NCC GC về điều chuyển: Điều phối thành phẩm hay Chuyên viên Quản lý hồ sơ SX và Dữ liệu NCC GC?</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -541,29 +538,24 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>- [Chị Ngân · V3 · C4] Trưởng phòng (Quản lý sản xuất) chịu trách nhiệm cuối quyết định duyệt cho đơn hàng triển khai (kể cả trường hợp duyệt trước bổ sung sau)
-- [Trưởng nhóm Quản lý dữ liệu · V6 · C1] Phòng Kinh doanh là đơn vị xem xét và quyết định việc tiếp tục triển khai hoặc tạm dừng đơn hàng khi kiểm tra điều kiện có vướng mắc; Điều phối thành phẩm phối hợp kiểm tra và thông báo</t>
+          <t>1. Phiếu yêu cầu điều chuyển nguyên liệu được lập và gửi cho Điều phối thành phẩm để gửi tiếp cho NCC GC phối hợp xuất và điều chuyển  (Chuyên viên Điều phối nguyên liệu/bán thành phẩm)
+2. Chuyên viên Quản lý hồ sơ sản xuất và Dữ liệu NCC GC làm đầu mối giao dịch với NCC GC về việc điều chuyển nguyên liệu  (Trưởng nhóm Điều phối)</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Cả hai là as-is. Trưởng phòng nói Trưởng phòng quyết cuối, kể cả duyệt trước bổ sung sau. Trưởng nhóm QLDL nói KD quyết.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Trưởng nhóm Điều phối</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>M03</t>
-        </is>
+      <c r="A4" s="2" t="n">
+        <v>3</v>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Chi phí phát sinh của một đơn gia công hiện có phải xin duyệt không, ai duyệt, ngưỡng bao nhiêu?</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -571,29 +563,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>- [Trưởng nhóm Điều phối · V2 · C4] Quản lý sản xuất là người quyết định cuối cùng (cho duyệt trước bổ sung sau hoặc tạm ngưng đơn) dựa trên dữ liệu kiểm tra từ các nhóm nội bộ; Trưởng nhóm Điều phối cập nhật tiến độ lại cho Kinh doanh
-- [Trưởng nhóm Quản lý dữ liệu · V6 · C1] Phòng Kinh doanh là đơn vị xem xét và quyết định việc tiếp tục triển khai hoặc tạm dừng đơn hàng khi kiểm tra điều kiện có vướng mắc; Điều phối thành phẩm phối hợp kiểm tra và thông báo</t>
+          <t>1. Không áp dụng phê duyệt chi phí hoặc vượt ngân sách dự toán đơn hàng do công ty hiện không có quỹ chi phí và ngân sách dự toán  (Chị Ngân)
+2. Chi phí phát sinh ngoài ngân sách sản xuất phải trình Giám đốc phụ trách và ghi kèm tên công ty tương ứng để phê duyệt (áp dụng cho 12 công ty thuộc Group)  (Giám đốc)</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Cả hai là as-is, độ tin cao. Hai trưởng nhóm nói hai người quyết khác nhau.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Giám đốc, Trưởng phòng Sản xuất, Phòng Tài chính Kế toán</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>M04</t>
-        </is>
+      <c r="A5" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Xác nhận đây là hai việc khác nhau: duyệt hợp đồng NCC mới đi theo tệp quy trình; duyệt chi phí theo câu trả lời ở M12.?</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -601,29 +588,24 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>- [Chị Ngân · V3 · C4] Trưởng phòng (Quản lý sản xuất) chịu trách nhiệm cuối quyết định duyệt cho đơn hàng triển khai (kể cả trường hợp duyệt trước bổ sung sau)
-- [Chuyên viên Điều phối vật tư bao bì · V3 · C3] Trưởng phòng sản xuất hoặc Phòng Kinh doanh quyết định cuối cùng về việc duyệt tiếp hay dừng đơn khi tồn kho VTBB không đủ hoặc không kịp tiến độ đơn hàng</t>
+          <t>1. Duyệt hợp đồng NCC GC mới lần lượt qua Pháp lý -&gt; P. TCKT -&gt; Giám đốc ký duyệt  (QUY TRÌNH SẢN XUẤT 09.07.2026 (2).xlsx)
+2. Không áp dụng phê duyệt chi phí hoặc vượt ngân sách dự toán đơn hàng do công ty hiện không có quỹ chi phí và ngân sách dự toán  (Chị Ngân)</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Chuyên viên VTBB nói Trưởng phòng hoặc KD, chưa phân định khi hai bên bất đồng.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Trưởng phòng Sản xuất</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>M05</t>
-        </is>
+      <c r="A6" s="2" t="n">
+        <v>5</v>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Mỗi ngày nhận bao nhiêu yêu cầu từ KD, và mỗi tuần có bao nhiêu đơn thật sự gửi NCC GC?</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -631,29 +613,24 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C2] Phòng Kinh doanh xem xét và quyết định phương án duyệt hoặc hoãn đơn hàng khi NL/BTP không đủ hoặc không kịp tiến độ
-- [Chuyên viên Điều phối vật tư bao bì · V3 · C3] Trưởng phòng sản xuất hoặc Phòng Kinh doanh quyết định cuối cùng về việc duyệt tiếp hay dừng đơn khi tồn kho VTBB không đủ hoặc không kịp tiến độ đơn hàng</t>
+          <t>1. Tiếp nhận khoảng 10 đến 15 đơn hàng một ngày từ Phòng Kinh doanh (bao gồm cả các đơn hàng dự trù trước). Chuyên viên VTBB V3 C1 cũng nói 10 đến 15 đơn mỗi ngày.  (Chuyên viên Điều phối sản xuất)
+2. Trung bình khoảng 15 đơn/tuần cho 3 loại: đơn thành phẩm, đơn bán thành phẩm, đơn xử lý lại. Chuyên viên Giá vốn V2 C1 cũng nói khoảng 15 đơn mỗi tuần.  (Trưởng nhóm Điều phối)</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Chuyên viên NL/BTP nói KD quyết khi thiếu NL/BTP. Chuyên viên VTBB nói Trưởng phòng hoặc KD khi thiếu VTBB.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Trưởng nhóm Điều phối, Chuyên viên Điều phối sản xuất</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>M06</t>
-        </is>
+      <c r="A7" s="2" t="n">
+        <v>6</v>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Hạn mức 3 triệu và 5 triệu trong tệp quy trình thanh toán có đang áp cho chi phí của phòng Sản xuất không? Giám đốc phụ trách và Giám đốc điều hành có phải một người?</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -661,29 +638,24 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>- [Chị Ngân · V3 · C4] Trưởng phòng (Quản lý sản xuất) chịu trách nhiệm cuối quyết định duyệt cho đơn hàng triển khai (kể cả trường hợp duyệt trước bổ sung sau)
-- [Trưởng nhóm Quản lý dữ liệu · V3 · C1] Nhân sự phụ trách thông báo trực tiếp cho Phòng Kinh doanh và Quản lý để xem xét, quyết định tiếp tục triển khai hoặc tạm dừng đơn hàng khi điều kiện triển khai chưa đáp ứng</t>
+          <t>1. Không áp dụng phê duyệt chi phí hoặc vượt ngân sách dự toán (Giám đốc V1 C1 lại nói phải trình Giám đốc phụ trách).  (Chị Ngân)
+2. Trưởng bộ phận duyệt tối đa 3 triệu/lần (hạn mức 10 triệu/tháng); Quản lý thương hiệu duyệt tối đa 5 triệu/lần; vượt mức do Giám đốc điều hành duyệt.  (Bản sao của QUY TRINH THANH TOAN V1- 7.11.2025.xlsx)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Trưởng phòng nói mình quyết. Trưởng nhóm QLDL (vòng 3) nói báo cả KD và Quản lý cùng xem xét.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Giám đốc, Phòng Tài chính Kế toán</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>M07</t>
-        </is>
+      <c r="A8" s="2" t="n">
+        <v>7</v>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Phiếu phối trộn và phiếu điều chuyển nguyên liệu có gửi thẳng cho Kho không? Nếu khác nhau thì mỗi loại gửi ai?</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -691,29 +663,24 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C2] Phòng Kinh doanh xem xét và quyết định phương án duyệt hoặc hoãn đơn hàng khi NL/BTP không đủ hoặc không kịp tiến độ
-- [Trưởng nhóm Quản lý dữ liệu · V3 · C1] Nhân sự phụ trách thông báo trực tiếp cho Phòng Kinh doanh và Quản lý để xem xét, quyết định tiếp tục triển khai hoặc tạm dừng đơn hàng khi điều kiện triển khai chưa đáp ứng</t>
+          <t>1. Phiếu yêu cầu phối trộn hoặc điều chuyển nguyên liệu gửi Phòng Kinh doanh, Bộ phận Kho và Nhà gia công.  (Chuyên viên Điều phối nguyên liệu/bán thành phẩm)
+2. Bộ phận Sản xuất không gửi trực tiếp Phiếu điều chuyển nguyên liệu cho Kho, mà gửi Điều phối thành phẩm để yêu cầu NCC GC phối hợp xuất điều chuyển.  (Chuyên viên Điều phối nguyên liệu/bán thành phẩm)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>KD quyết, so với KD và Quản lý cùng quyết.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Chuyên viên Điều phối nguyên liệu/bán thành phẩm</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>M08</t>
-        </is>
+      <c r="A9" s="2" t="n">
+        <v>8</v>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Làm ra gì, giao cho ai, qua kênh nào / Ai làm
-(Quản lý đơn hàng SX gia công · Chuẩn bị nguồn lực và hoàn thiện điều kiện đặt hàng)</t>
+          <t>Điều phối thành phẩm và Chuyên viên Điều phối sản xuất có phải một vị trí? Đơn sai quy cách do KD ghi sai thì ai chịu?</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -721,29 +688,24 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C5] Phiếu yêu cầu điều chuyển nguyên liệu được lập và gửi cho Điều phối thành phẩm để gửi tiếp cho NCC GC phối hợp xuất và điều chuyển
-- [Trưởng nhóm Điều phối · V4 · C1] Chuyên viên Quản lý hồ sơ sản xuất và Dữ liệu NCC GC làm đầu mối giao dịch với NCC GC về việc điều chuyển nguyên liệu</t>
+          <t>1. Điều phối thành phẩm chịu trách nhiệm đảm bảo tính đầy đủ của thông tin, Phòng Kinh doanh chịu trách nhiệm đảm bảo tính chính xác của đơn đặt hàng.  (Trưởng nhóm Điều phối)
+2. Chuyên viên Điều phối sản xuất chịu trách nhiệm cuối nếu đơn hàng bị sót thông tin hoặc sai quy cách.  (Chị Ngân)</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Nhận định MIC: Chuyên viên NL/BTP nói phiếu đi qua Điều phối thành phẩm; Trưởng nhóm Điều phối nói Điều phối thành phẩm chỉ nhận thông tin đủ hàng, giao dịch với NCC GC do nhóm Quản lý dữ liệu làm. Thêm nguồn thứ ba: Chuyên viên Điều phối sản xuất V3 C2 nói mình nhận phiếu điều chuyển để làm việc với NCC GC.
-Đề nghị chốt: Phiếu yêu cầu điều chuyển nguyên liệu gửi cho ai, và ai là đầu mối làm việc với NCC GC về điều chuyển: Điều phối thành phẩm hay Chuyên viên Quản lý hồ sơ SX và Dữ liệu NCC GC?
-Người chốt đề nghị: Trưởng nhóm Điều phối</t>
+          <t>Người nên chốt: Trưởng phòng Sản xuất</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>M09</t>
-        </is>
+      <c r="A10" s="2" t="n">
+        <v>9</v>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Hàng nhận về bị lỗi: ai quyết phương án cuối? Có tách theo lúc phát hiện (tại NCC hay đã về kho) không?</t>
         </is>
       </c>
       <c r="C10" s="2" t="n">
@@ -751,29 +713,24 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C2] Phòng Kinh doanh xem xét và quyết định phương án duyệt hoặc hoãn đơn hàng khi NL/BTP không đủ hoặc không kịp tiến độ
-- [Chuyên viên Pháp lý - Xử lý sự cố · V3 · C1] Quản lý sản xuất là người quyết định cuối cùng việc duyệt cho đơn hàng triển khai hay không khi hồ sơ pháp lý chưa đạt hoặc chưa đủ</t>
+          <t>1. Trưởng nhóm Điều phối quyết định phương án xử lý cuối cùng sau khi tổng hợp ý kiến từ NCC GC, các bộ phận liên quan và Kinh doanh.  (Trưởng nhóm Điều phối)
+2. Trưởng nhóm Quản lý dữ liệu phê duyệt phương án trong thẩm quyền; ngoài quy trình, vượt thẩm quyền hoặc có rủi ro thì Trưởng phòng quyết định.  (Chuyên viên Pháp lý - Xử lý sự cố)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>KD quyết khi thiếu NL/BTP, so với Quản lý sản xuất quyết khi hồ sơ pháp lý chưa đạt. Hai câu có thể nói về hai loại vướng mắc khác nhau.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Trưởng phòng Sản xuất</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>M10</t>
-        </is>
+      <c r="A11" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Bản quy trình chuẩn hiện hành là bản nào: 6 bước hay 7 bước?</t>
         </is>
       </c>
       <c r="C11" s="2" t="n">
@@ -781,29 +738,24 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C2] Phòng Kinh doanh xem xét và quyết định phương án duyệt hoặc hoãn đơn hàng khi NL/BTP không đủ hoặc không kịp tiến độ
-- [Chị Ngân · V3 · C4] Trưởng phòng (Quản lý sản xuất) chịu trách nhiệm cuối quyết định duyệt cho đơn hàng triển khai (kể cả trường hợp duyệt trước bổ sung sau)</t>
+          <t>1. Quy trình quan trọng nhất gồm 6 bước từ tiếp nhận đơn đến hoàn thiện chứng từ thanh lý.  (Chị Ngân)
+2. Gồm 7 bước: tiếp nhận và xử lý dữ liệu, kiểm tra thông tin, gửi đơn NCC, nhập kho và nhận hóa đơn, theo dõi nhận hàng, kiểm tra mẫu gửi Lab, lập chứng từ.  (QUY TRÌNH SẢN XUẤT 09.07.2026 (1).xlsx)</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>KD quyết, so với Trưởng phòng quyết.
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Trưởng phòng Sản xuất</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>M11</t>
-        </is>
+      <c r="A12" s="2" t="n">
+        <v>11</v>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Kiểm tra điều kiện triển khai đơn hàng)</t>
+          <t>Với từng công ty, ai duyệt kết quả chọn NCC mới và ai ký hợp đồng?</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
@@ -811,29 +763,24 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C2] Phòng Kinh doanh xem xét và quyết định phương án duyệt hoặc hoãn đơn hàng khi NL/BTP không đủ hoặc không kịp tiến độ
-- [Trưởng nhóm Điều phối · V2 · C4] Quản lý sản xuất là người quyết định cuối cùng (cho duyệt trước bổ sung sau hoặc tạm ngưng đơn) dựa trên dữ liệu kiểm tra từ các nhóm nội bộ; Trưởng nhóm Điều phối cập nhật tiến độ lại cho Kinh doanh</t>
+          <t>1. Duyệt hợp đồng NCC GC mới lần lượt qua Pháp lý -&gt; P. TCKT -&gt; Giám đốc ký duyệt.  (QUY TRÌNH SẢN XUẤT 09.07.2026 (2).xlsx)
+2. Hợp đồng và bảng giá với NCC mới bắt buộc trình Đại diện pháp luật của Công ty ký duyệt. Giám đốc V1 C2: Giám đốc phụ trách công ty tương ứng duyệt bằng văn bản.  (Giám đốc)</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>KD quyết, so với Quản lý sản xuất quyết (Trưởng nhóm Điều phối chỉ báo lại tiến độ cho KD).
-Đề nghị chốt: Khi đơn hàng không đủ điều kiện triển khai, ai quyết cuối cho đi tiếp hay dừng? Đề xuất chia theo loại vướng mắc: pháp lý và cung ứng nội bộ do Trưởng phòng quyết; dời ngày giao hoặc hủy đơn với khách do Phòng Kinh doanh quyết; hai bên không thống nhất thì Giám đốc. Xác nhận hoặc sửa.
-Người chốt đề nghị: Trưởng phòng Sản xuất, Giám đốc (hỏi ý Phòng Kinh doanh)</t>
+          <t>Người nên chốt: Giám đốc</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>M12</t>
-        </is>
+      <c r="A13" s="2" t="n">
+        <v>12</v>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Việc nào phải xin duyệt, ai duyệt, ngưỡng nào
-(Tổng quan phòng · Duyệt và ngưỡng)</t>
+          <t>KD đang hứa ngày giao theo bảng nào? Bảng nào là bảng đúng?</t>
         </is>
       </c>
       <c r="C13" s="2" t="n">
@@ -841,29 +788,24 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>- [Chị Ngân · V2 · C2] Không áp dụng phê duyệt chi phí hoặc vượt ngân sách dự toán đơn hàng do công ty hiện không có quỹ chi phí và ngân sách dự toán
-- [Giám đốc · V1 · C1] Chi phí phát sinh ngoài ngân sách sản xuất phải trình Giám đốc phụ trách và ghi kèm tên công ty tương ứng để phê duyệt (áp dụng cho 12 công ty thuộc Group)</t>
+          <t>1. Thời gian sản xuất một đơn tại NCC Hà Long: 15, 10 hoặc 7 ngày tùy ai cấp BTP và VTBB.  (Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx)
+2. NCC Hà Long: thời gian 5-14 ngày.  (QUY TRÌNH SẢN XUẤT 09.07.2026 (1).xlsx)</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Trưởng phòng nói không có ngân sách dự toán nên không duyệt chi phí phát sinh. Giám đốc nói chi phí ngoài ngân sách phải trình Giám đốc phụ trách công ty tương ứng. Có thể hai câu nói về hai việc: không có ngân sách theo đơn hàng, nhưng chi phí phát sinh vẫn phải xin duyệt. Xem thêm L02.
-Đề nghị chốt: Chi phí phát sinh của một đơn gia công hiện có phải xin duyệt không, ai duyệt, ngưỡng bao nhiêu?
-Người chốt đề nghị: Giám đốc, Trưởng phòng Sản xuất, Phòng Tài chính Kế toán</t>
+          <t>Người nên chốt: Trưởng nhóm Điều phối</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>M13</t>
-        </is>
+      <c r="A14" s="2" t="n">
+        <v>13</v>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Việc nào phải xin duyệt, ai duyệt, ngưỡng nào
-(Tổng quan phòng · Duyệt và ngưỡng)</t>
+          <t>Đây là một bộ trạng thái hay hai bộ? Liệt kê tên từng trạng thái.?</t>
         </is>
       </c>
       <c r="C14" s="2" t="n">
@@ -871,29 +813,24 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>- [QUY TRÌNH SẢN XUẤT 09.07.2026 (2).xlsx · sheet 1. QT LÀM VIỆC VỚI NCC MỚI] Duyệt hợp đồng NCC GC mới lần lượt qua Pháp lý -&gt; P. TCKT -&gt; Giám đốc ký duyệt
-- [Chị Ngân · V2 · C2] Không áp dụng phê duyệt chi phí hoặc vượt ngân sách dự toán đơn hàng do công ty hiện không có quỹ chi phí và ngân sách dự toán</t>
+          <t>1. Tiến độ đơn hàng theo dõi qua 6 trạng thái điều phối.  (Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx)
+2. Quy trình điều phối theo dõi 7 trạng thái nhập xuất.  (Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx)</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Trạng thái trên MIC: đã hỏi lại. Hai câu nói về hai việc khác nhau (duyệt hợp đồng NCC mới và duyệt chi phí), nên nhiều khả năng không mâu thuẫn thật. Điểm thật cần chốt nằm ở L07.
-Đề nghị chốt: Xác nhận đây là hai việc khác nhau: duyệt hợp đồng NCC mới đi theo tệp quy trình; duyệt chi phí theo câu trả lời ở M12.
-Người chốt đề nghị: Trưởng phòng Sản xuất</t>
+          <t>Người nên chốt: Trưởng nhóm Điều phối</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>L01</t>
-        </is>
+      <c r="A15" s="2" t="n">
+        <v>14</v>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>Bao lâu một lần (số đơn)
-(Quản lý đơn hàng SX gia công · Tiếp nhận / Kiểm tra điều kiện)</t>
+          <t>Khi nhận thành phẩm, Kho kiểm gì, Lab kiểm gì? Kết quả của bên nào quyết định hàng được nhập kho?</t>
         </is>
       </c>
       <c r="C15" s="2" t="n">
@@ -901,29 +838,24 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối sản xuất · V2 · C1] Tiếp nhận khoảng 10 đến 15 đơn hàng một ngày từ Phòng Kinh doanh (bao gồm cả các đơn hàng dự trù trước). Chuyên viên VTBB V3 C1 cũng nói 10 đến 15 đơn mỗi ngày.
-- [Trưởng nhóm Điều phối · V4 · C2] Trung bình khoảng 15 đơn/tuần cho 3 loại: đơn thành phẩm, đơn bán thành phẩm, đơn xử lý lại. Chuyên viên Giá vốn V2 C1 cũng nói khoảng 15 đơn mỗi tuần.</t>
+          <t>1. Lab nội bộ kiểm mẫu thành phẩm khi nhận hàng từ NCC GC: ngoại dạng, màu sắc, trọng lượng; kiểm hàm lượng chỉ khi có yêu cầu hoặc sự cố.  (Trưởng nhóm Điều phối)
+2. Biểu mẫu Kết quả KCS Kho dùng theo dõi quy cách ngoại quan, phụ kiện và chứng từ khi nhận thành phẩm.  (Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Lệch khoảng 5 lần. Giả thuyết: hai nhóm đếm hai thứ khác nhau, một bên đếm mọi yêu cầu KD gửi vào (gồm đơn dự trù), một bên đếm đơn thật sự đi duyệt giá và gửi NCC.
-Đề nghị chốt: Mỗi ngày nhận bao nhiêu yêu cầu từ KD, và mỗi tuần có bao nhiêu đơn thật sự gửi NCC GC?
-Người chốt đề nghị: Trưởng nhóm Điều phối, Chuyên viên Điều phối sản xuất</t>
+          <t>Người nên chốt: Trưởng nhóm Điều phối, Kho, Lab</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>L02</t>
-        </is>
+      <c r="A16" s="2" t="n">
+        <v>15</v>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Việc nào phải xin duyệt, ai duyệt, ngưỡng nào
-(Tổng quan phòng · Duyệt và ngưỡng)</t>
+          <t>Ai đang giữ vị trí Chuyên viên Pháp lý - Xử lý sự cố? Người trả lời khảo sát ở vai này là ai?</t>
         </is>
       </c>
       <c r="C16" s="2" t="n">
@@ -931,29 +863,24 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>- [Chị Ngân · V2 · C2] Không áp dụng phê duyệt chi phí hoặc vượt ngân sách dự toán (Giám đốc V1 C1 lại nói phải trình Giám đốc phụ trách).
-- [Bản sao của QUY TRINH THANH TOAN V1- 7.11.2025.xlsx · sheet Form DE XUAT MUA HANG] Trưởng bộ phận duyệt tối đa 3 triệu/lần (hạn mức 10 triệu/tháng); Quản lý thương hiệu duyệt tối đa 5 triệu/lần; vượt mức do Giám đốc điều hành duyệt.</t>
+          <t>1. Chuyên viên Pháp lý - Xử lý sự cố: Trần Ngọc Huỳnh (lead), Nguyễn Ngọc Bảo Thi.  (Ảnh sơ đồ tổ chức)
+2. Chuyên viên Pháp lý - Xử lý sự cố: Trần Ngọc Huỳnh kiêm nhiệm và một nhân viên tên Thơ.  (Danh sách vị trí trên MIC)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Ba nguồn, ba kiểu. MIC chỉ so cặp Trưởng phòng và Giám đốc (M12), chưa so với tệp có hạn mức. Còn một chỗ lệch nhỏ: Giám đốc phụ trách và Giám đốc điều hành có phải một người không.
-Đề nghị chốt: Hạn mức 3 triệu và 5 triệu trong tệp quy trình thanh toán có đang áp cho chi phí của phòng Sản xuất không? Giám đốc phụ trách và Giám đốc điều hành có phải một người?
-Người chốt đề nghị: Giám đốc, Phòng Tài chính Kế toán</t>
+          <t>Người nên chốt: Trưởng phòng Sản xuất</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>L03</t>
-        </is>
+      <c r="A17" s="2" t="n">
+        <v>16</v>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>Phiếu điều chuyển nguyên liệu gửi cho ai
-(Quản lý đơn hàng SX gia công · Chuẩn bị nguồn lực)</t>
+          <t>Chuyên viên Điều phối NL/BTP báo cáo trực tiếp cho ai? Nhân sự có tên ở hai nhóm có kiêm nhiệm không?</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
@@ -961,291 +888,18 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V1 · C2] Phiếu yêu cầu phối trộn hoặc điều chuyển nguyên liệu gửi Phòng Kinh doanh, Bộ phận Kho và Nhà gia công.
-- [Chuyên viên Điều phối nguyên liệu/bán thành phẩm · V2 · C5] Bộ phận Sản xuất không gửi trực tiếp Phiếu điều chuyển nguyên liệu cho Kho, mà gửi Điều phối thành phẩm để yêu cầu NCC GC phối hợp xuất điều chuyển.</t>
+          <t>1. Chuyên viên Điều phối NL/BTP báo cáo Trưởng nhóm Điều phối. Cùng một nhân sự có tên ở cả nhóm Điều phối sản xuất và nhóm Điều phối NL/BTP.  (Ảnh sơ đồ tổ chức)
+2. Chuyên viên Điều phối NL/BTP phản hồi chưa xác định rõ Trưởng nhóm Điều phối có phải quản lý trực tiếp hay không.  (Lỗ hổng trên MIC (mức cao))</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Cùng một người nói hai ý ở hai vòng. Giả thuyết: phiếu phối trộn gửi Kho, phiếu điều chuyển thì không.
-Đề nghị chốt: Phiếu phối trộn và phiếu điều chuyển nguyên liệu có gửi thẳng cho Kho không? Nếu khác nhau thì mỗi loại gửi ai?
-Người chốt đề nghị: Chuyên viên Điều phối nguyên liệu/bán thành phẩm</t>
+          <t>Người nên chốt: Trưởng phòng Sản xuất</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr"/>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>L04</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Ai chịu trách nhiệm cuối
-(Quản lý đơn hàng SX gia công · Tiếp nhận và kiểm tra yêu cầu đặt hàng)</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>- [Trưởng nhóm Điều phối · V2 · C3] Điều phối thành phẩm chịu trách nhiệm đảm bảo tính đầy đủ của thông tin, Phòng Kinh doanh chịu trách nhiệm đảm bảo tính chính xác của đơn đặt hàng.
-- [Chị Ngân · V3 · C3] Chuyên viên Điều phối sản xuất chịu trách nhiệm cuối nếu đơn hàng bị sót thông tin hoặc sai quy cách.</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Nếu Điều phối thành phẩm và Chuyên viên Điều phối sản xuất là một vị trí thì chỉ lệch ở phần trách nhiệm của KD. Hai tên gọi đang dùng lẫn.
-Đề nghị chốt: Điều phối thành phẩm và Chuyên viên Điều phối sản xuất có phải một vị trí? Đơn sai quy cách do KD ghi sai thì ai chịu?
-Người chốt đề nghị: Trưởng phòng Sản xuất</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="inlineStr"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>L05</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Ai quyết phương án khi hàng lỗi
-(Quản lý đơn hàng SX gia công · Nhận hàng và xử lý sai lệch / Xử lý sự cố)</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>- [Trưởng nhóm Điều phối · V4 · C4] Trưởng nhóm Điều phối quyết định phương án xử lý cuối cùng sau khi tổng hợp ý kiến từ NCC GC, các bộ phận liên quan và Kinh doanh.
-- [Chuyên viên Pháp lý - Xử lý sự cố · V5 · C3] Trưởng nhóm Quản lý dữ liệu phê duyệt phương án trong thẩm quyền; ngoài quy trình, vượt thẩm quyền hoặc có rủi ro thì Trưởng phòng quyết định.</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Hai trưởng nhóm khác nhau cùng được nói là người quyết. Giả thuyết: Trưởng nhóm Điều phối quyết khi lỗi phát hiện lúc nhận hàng tại NCC, Trưởng nhóm QLDL quyết khi đã thành sự cố.
-Đề nghị chốt: Hàng nhận về bị lỗi: ai quyết phương án cuối? Có tách theo lúc phát hiện (tại NCC hay đã về kho) không?
-Người chốt đề nghị: Trưởng phòng Sản xuất</t>
-        </is>
-      </c>
-      <c r="F19" s="3" t="inlineStr"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>L06</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Các bước theo thứ tự
-(Quản lý đơn hàng SX gia công · Mức quy trình)</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>- [Chị Ngân · V1 · C4] Quy trình quan trọng nhất gồm 6 bước từ tiếp nhận đơn đến hoàn thiện chứng từ thanh lý.
-- [QUY TRÌNH SẢN XUẤT 09.07.2026 (1).xlsx · sheet 4. QT QL ĐƠN HÀNG SX GC] Gồm 7 bước: tiếp nhận và xử lý dữ liệu, kiểm tra thông tin, gửi đơn NCC, nhập kho và nhận hóa đơn, theo dõi nhận hàng, kiểm tra mẫu gửi Lab, lập chứng từ.</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Số bước và tên bước khác nhau giữa câu trả lời và tệp quy trình. MIC đang dựng theo 6 bước.
-Đề nghị chốt: Bản quy trình chuẩn hiện hành là bản nào: 6 bước hay 7 bước?
-Người chốt đề nghị: Trưởng phòng Sản xuất</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>L07</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Ai ký hợp đồng NCC GC mới
-(Làm việc với NCC GC mới · Soạn hợp đồng / Hoàn thiện)</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D21" s="2" t="inlineStr">
-        <is>
-          <t>- [QUY TRÌNH SẢN XUẤT 09.07.2026 (2).xlsx · sheet 1. QT LÀM VIỆC VỚI NCC MỚI] Duyệt hợp đồng NCC GC mới lần lượt qua Pháp lý -&gt; P. TCKT -&gt; Giám đốc ký duyệt.
-- [Giám đốc · V2 · C2] Hợp đồng và bảng giá với NCC mới bắt buộc trình Đại diện pháp luật của Công ty ký duyệt. Giám đốc V1 C2: Giám đốc phụ trách công ty tương ứng duyệt bằng văn bản.</t>
-        </is>
-      </c>
-      <c r="E21" s="2" t="inlineStr">
-        <is>
-          <t>Tập đoàn có 12 công ty. Giám đốc ký, Giám đốc phụ trách và Đại diện pháp luật có thể là những người khác nhau ở từng công ty.
-Đề nghị chốt: Với từng công ty, ai duyệt kết quả chọn NCC mới và ai ký hợp đồng?
-Người chốt đề nghị: Giám đốc</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>L08</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>Toàn trình mất bao lâu
-(Quản lý đơn hàng SX gia công · Mức quy trình)</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D22" s="2" t="inlineStr">
-        <is>
-          <t>- [Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx · sheet Data số ngày cập nhật cho KD] Thời gian sản xuất một đơn tại NCC Hà Long: 15, 10 hoặc 7 ngày tùy ai cấp BTP và VTBB.
-- [QUY TRÌNH SẢN XUẤT 09.07.2026 (1).xlsx · sheet 17. TT NCC GC] NCC Hà Long: thời gian 5-14 ngày.</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Hai bảng cùng nói về một NCC nhưng khác số.
-Đề nghị chốt: KD đang hứa ngày giao theo bảng nào? Bảng nào là bảng đúng?
-Người chốt đề nghị: Trưởng nhóm Điều phối</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>L09</t>
-        </is>
-      </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>Số trạng thái theo dõi đơn
-(Công cụ, tài liệu)</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>- [Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx · sheet họp07.10] Tiến độ đơn hàng theo dõi qua 6 trạng thái điều phối.
-- [Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx · sheet NHẬP-XUẤT TP] Quy trình điều phối theo dõi 7 trạng thái nhập xuất.</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Hai sheet trong cùng một tệp. Có thể là hai bộ trạng thái khác nhau (điều phối và nhập xuất).
-Đề nghị chốt: Đây là một bộ trạng thái hay hai bộ? Liệt kê tên từng trạng thái.
-Người chốt đề nghị: Trưởng nhóm Điều phối</t>
-        </is>
-      </c>
-      <c r="F23" s="3" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>L10</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>Ai kiểm chất lượng thành phẩm khi nhận
-(Quản lý đơn hàng SX gia công · Nhận hàng)</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>- [Trưởng nhóm Điều phối · V2 · C7] Lab nội bộ kiểm mẫu thành phẩm khi nhận hàng từ NCC GC: ngoại dạng, màu sắc, trọng lượng; kiểm hàm lượng chỉ khi có yêu cầu hoặc sự cố.
-- [Bản sao của ĐIỀU PHỒI THÀNH PHẨM (NHÁP).xlsx · sheet Kết quả KCS Kho Dr.Xanh] Biểu mẫu Kết quả KCS Kho dùng theo dõi quy cách ngoại quan, phụ kiện và chứng từ khi nhận thành phẩm.</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Có thể cả Lab và Kho cùng kiểm, mỗi bên một phần. Cần biết kết quả của bên nào thì hàng mới được nhập kho dùng được.
-Đề nghị chốt: Khi nhận thành phẩm, Kho kiểm gì, Lab kiểm gì? Kết quả của bên nào quyết định hàng được nhập kho?
-Người chốt đề nghị: Trưởng nhóm Điều phối, Kho, Lab</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>L11</t>
-        </is>
-      </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>Ai đang giữ vị trí Chuyên viên Pháp lý - Xử lý sự cố
-(Bộ máy)</t>
-        </is>
-      </c>
-      <c r="C25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>- [Ảnh sơ đồ tổ chức · tr. 1] Chuyên viên Pháp lý - Xử lý sự cố: Trần Ngọc Huỳnh (lead), Nguyễn Ngọc Bảo Thi.
-- [Danh sách vị trí trên MIC] Chuyên viên Pháp lý - Xử lý sự cố: Trần Ngọc Huỳnh kiêm nhiệm và một nhân viên tên Thơ.</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Mới phát hiện khi đọc lại ngày 24/10. Tên nhân viên thứ hai khác nhau. Nếu Trưởng nhóm QLDL đang kiêm vị trí này thì hai vai trả lời khác nhau ở câu ai quyết cuối (M09 so với M02).
-Đề nghị chốt: Ai đang giữ vị trí Chuyên viên Pháp lý - Xử lý sự cố? Người trả lời khảo sát ở vai này là ai?
-Người chốt đề nghị: Trưởng phòng Sản xuất</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>L12</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>Tuyến báo cáo của Chuyên viên Điều phối NL/BTP
-(Bộ máy)</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>- [Ảnh sơ đồ tổ chức · tr. 1] Chuyên viên Điều phối NL/BTP báo cáo Trưởng nhóm Điều phối. Cùng một nhân sự có tên ở cả nhóm Điều phối sản xuất và nhóm Điều phối NL/BTP.
-- [Lỗ hổng trên MIC (mức cao)] Chuyên viên Điều phối NL/BTP phản hồi chưa xác định rõ Trưởng nhóm Điều phối có phải quản lý trực tiếp hay không.</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Có thể do kiêm nhiệm hai vị trí, và Trưởng nhóm Điều phối đang do Trưởng phòng kiêm nhiệm.
-Đề nghị chốt: Chuyên viên Điều phối NL/BTP báo cáo trực tiếp cho ai? Nhân sự có tên ở hai nhóm có kiêm nhiệm không?
-Người chốt đề nghị: Trưởng phòng Sản xuất</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:F26"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>